<commit_message>
hidden and show product
</commit_message>
<xml_diff>
--- a/data/affiliate/picks.xlsx
+++ b/data/affiliate/picks.xlsx
@@ -1333,7 +1333,7 @@
     <row r="17" ht="18" customHeight="1">
       <c r="A17" t="inlineStr">
         <is>
-          <t>ai_calculator</t>
+          <t>ai_calculator_cpu</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -1343,20 +1343,20 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>VGA (การ์ดแสดงผล) MSI GEFORCE RTX 5090 32G GAMING TRIO OC - 32GB GDDR7</t>
+          <t>CPU (ซีพียู) AMD RYZEN 9 7950X 4.5 GHz (SOCKET AM5) (ระบบระบายความร้อนไม่รวมอยู่ในสินค้า) -3 YEARS</t>
         </is>
       </c>
       <c r="E17" t="n">
-        <v>169700</v>
+        <v>22700</v>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/2BD1GnZPSV</t>
+          <t>https://s.shopee.co.th/2qSiUqO1NA</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>https://down-zl-th.img.susercontent.com/th-11134207-7ra0m-mbet1fh1hbnaa6.webp</t>
+          <t>https://down-ws-th.img.susercontent.com/th-11134207-7rasd-m8x801x6gycuda.webp</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
@@ -1364,24 +1364,19 @@
           <t>Shopee</t>
         </is>
       </c>
-      <c r="J17" t="inlineStr">
-        <is>
-          <t>ขายดี</t>
-        </is>
-      </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>JIB Official Store</t>
+          <t>mcwinner</t>
         </is>
       </c>
       <c r="L17" t="n">
-        <v>1</v>
+        <v>19</v>
       </c>
     </row>
     <row r="18" ht="18" customHeight="1">
       <c r="A18" t="inlineStr">
         <is>
-          <t>ai_calculator</t>
+          <t>ai_calculator_cpu</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -1391,20 +1386,20 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>คอมประกอบ GIGABYTE AITOP : Computer Set intel #i375 ULTRA 9 285K RTX5090 32GB GIGABYTE WINDFORCE (OC/D7) - A0172192</t>
+          <t>CPU (ซีพียู) AMD RYZEN 9 9950X - 16C 32T 4.3-5.7GHz (AMD SOCKET AM5) (ระบบระบายความร้อนไม่รวมอยู่ในสินค้า)</t>
         </is>
       </c>
       <c r="E18" t="n">
-        <v>301100</v>
+        <v>26500</v>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/1gGkfsbJTQ</t>
+          <t>https://s.shopee.co.th/2g9IIXOei9</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>https://down-zl-th.img.susercontent.com/th-11134207-81ztn-mq8t04g63tvx56.webp</t>
+          <t>https://down-ws-th.img.susercontent.com/th-11134207-7r991-m08fblrkcqfsb1.webp</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
@@ -1412,21 +1407,19 @@
           <t>Shopee</t>
         </is>
       </c>
-      <c r="J18" t="inlineStr">
-        <is>
-          <t>ขายดี</t>
-        </is>
-      </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>Advice Official Shop</t>
-        </is>
+          <t>JIB Official Store</t>
+        </is>
+      </c>
+      <c r="L18" t="n">
+        <v>6</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>ai_calculator</t>
+          <t>ai_calculator_cpu</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -1436,20 +1429,20 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>คอมประกอบพรีเมียม / 4K | Ryzen 9 9950X3D + RTX 5090 | DDR5 12GB 6000MHz / SSD 1TB | ชุดน้ำปิด</t>
+          <t>CPU (ซีพียู) AMD RYZEN 5 9600X - 6C 12T 3.9-5.4GHz (AMD SOCKET AM5) (ระบบระบายความร้อนไม่รวมอยู่ในสินค้า)</t>
         </is>
       </c>
       <c r="E19" t="n">
-        <v>236900</v>
+        <v>10500</v>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/1qaAsBag8T</t>
+          <t>https://s.shopee.co.th/3B5YtSMkhG</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>https://down-zl-th.img.susercontent.com/sg-11134275-821eo-mh0e5nskf7k86e.webp</t>
+          <t>https://down-ws-th.img.susercontent.com/th-11134207-7ras8-m7agd6ph9f744c.webp</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
@@ -1457,21 +1450,19 @@
           <t>Shopee</t>
         </is>
       </c>
-      <c r="J19" t="inlineStr">
-        <is>
-          <t>ขายดี</t>
-        </is>
-      </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>บริษัท มังกี้ อีทีซี. จำกัด</t>
-        </is>
+          <t>JIB Official Store</t>
+        </is>
+      </c>
+      <c r="L19" t="n">
+        <v>382</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>ai_calculator</t>
+          <t>ai_calculator_cpu</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -1481,20 +1472,20 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>GIGABYTE RTX5090 AORUS INFINITY 32GB GDDR7</t>
+          <t>CPU (ซีพียู) AMD RYZEN 9 9950X3D - 16C 32T 4.3-5.7GHz AMD SOCKET AM5 (ระบบระบายความร้อนไม่รวมอยู่ในสินค้า)</t>
         </is>
       </c>
       <c r="E20" t="n">
-        <v>288900</v>
+        <v>33000</v>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/1LduHGca9O</t>
+          <t>https://s.shopee.co.th/30m8h9NO2F</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>https://down-zl-th.img.susercontent.com/th-11134207-81zte-mpeku3c4tngscb.webp</t>
+          <t>https://down-ws-th.img.susercontent.com/th-11134207-7rasd-m8ylj449xemnd8.webp</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
@@ -1502,21 +1493,19 @@
           <t>Shopee</t>
         </is>
       </c>
-      <c r="J20" t="inlineStr">
-        <is>
-          <t>ขายดี</t>
-        </is>
-      </c>
       <c r="K20" t="inlineStr">
         <is>
-          <t>EXPERT MINES COMPANY LIMITED</t>
-        </is>
+          <t>JIB Official Store</t>
+        </is>
+      </c>
+      <c r="L20" t="n">
+        <v>6</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>ai_calculator</t>
+          <t>ai_calculator_cpu</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -1526,20 +1515,20 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>MSI RTX5090 SUPRIM SOC 32GB GDDR7</t>
+          <t>ซีพียู CPU: AMD - RYZEN 9 (9950X AM5)</t>
         </is>
       </c>
       <c r="E21" t="n">
-        <v>195500</v>
+        <v>29900</v>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/1VxKTZbwoR</t>
+          <t>https://s.shopee.co.th/3ViPI4LU1M</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>https://down-zl-th.img.susercontent.com/th-11134207-7ras8-m8fwept4cfgvaf.webp</t>
+          <t>https://down-ws-th.img.susercontent.com/th-11134275-7rasm-maw7h34vstcg33.webp</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
@@ -1547,24 +1536,19 @@
           <t>Shopee</t>
         </is>
       </c>
-      <c r="J21" t="inlineStr">
-        <is>
-          <t>ขายดี</t>
-        </is>
-      </c>
       <c r="K21" t="inlineStr">
         <is>
-          <t>EXPERT MINES COMPANY LIMITED</t>
+          <t>atSine Tech</t>
         </is>
       </c>
       <c r="L21" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>ai_calculator</t>
+          <t>ai_calculator_cpu</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -1574,20 +1558,20 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>VGA (การ์ดแสดงผล) ASUS ROG ASTRAL GEFORCE RTX 5090 32GB GDDR7 OC EDITION</t>
+          <t>CPU AMD AM5 RYZEN 9 9900X3D (NEXT) - A0169017</t>
         </is>
       </c>
       <c r="E22" t="n">
-        <v>180700</v>
+        <v>24200</v>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/1113sedqpM</t>
+          <t>https://s.shopee.co.th/3LOz5lM7ML</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>https://down-zl-th.img.susercontent.com/th-11134207-7ra0u-mb7sojhocgfq48.webp</t>
+          <t>https://down-ws-th.img.susercontent.com/th-11134275-7rasf-maw7gzrwpuo1b1.webp</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
@@ -1595,21 +1579,19 @@
           <t>Shopee</t>
         </is>
       </c>
-      <c r="J22" t="inlineStr">
-        <is>
-          <t>ขายดี</t>
-        </is>
-      </c>
       <c r="K22" t="inlineStr">
         <is>
-          <t>JIB Official Store</t>
-        </is>
+          <t>Advice Official Shop</t>
+        </is>
+      </c>
+      <c r="L22" t="n">
+        <v>4</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>ai_calculator</t>
+          <t>ai_calculator_cpu</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -1619,20 +1601,20 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>ASUS ROG ASTRAL GAMING GEFORCE RTX5090 OC EDITION /32GB GDDR7 (90YV0LW0-M0NA00)</t>
+          <t>CPU AMD AM5 RYZEN 9 9950X3D (NEXT) - A0168684</t>
         </is>
       </c>
       <c r="E23" t="n">
-        <v>180000</v>
+        <v>32200</v>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/1BKU4xdDUP</t>
+          <t>https://s.shopee.co.th/3qLFggKDLS</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>https://down-zl-th.img.susercontent.com/th-11134207-7rasb-m847by4n5tkec6.webp</t>
+          <t>https://down-ws-th.img.susercontent.com/th-11134275-7rasf-maw7gzrwpuo1b1.webp</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
@@ -1640,18 +1622,13 @@
           <t>Shopee</t>
         </is>
       </c>
-      <c r="J23" t="inlineStr">
-        <is>
-          <t>ขายดี</t>
-        </is>
-      </c>
       <c r="K23" t="inlineStr">
         <is>
-          <t>TECHNOCOM.OFFICIAL</t>
+          <t>Advice Official Shop</t>
         </is>
       </c>
       <c r="L23" t="n">
-        <v>2</v>
+        <v>11</v>
       </c>
     </row>
     <row r="24">
@@ -1665,22 +1642,27 @@
           <t>item</t>
         </is>
       </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>5090</t>
+        </is>
+      </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>ASUS RTX 5090 ระบบระบายความร้อนด้วยน้ำ Night God Wind Cooling Night God TUF ZTE PowerColor 5090 OC เวอร์ชันต่างประเทศ</t>
+          <t>VGA (การ์ดแสดงผล) MSI GEFORCE RTX 5090 32G GAMING TRIO OC - 32GB GDDR7</t>
         </is>
       </c>
       <c r="E24" t="n">
-        <v>337700</v>
+        <v>169700</v>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/gODU2f7VK</t>
+          <t>https://s.shopee.co.th/2BD1GnZPSV</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>https://down-zl-th.img.susercontent.com/sg-11134201-8260c-mk0ukmy20v7p69.webp</t>
+          <t>https://down-zl-th.img.susercontent.com/th-11134207-7ra0m-mbet1fh1hbnaa6.webp</t>
         </is>
       </c>
       <c r="I24" t="inlineStr">
@@ -1695,7 +1677,7 @@
       </c>
       <c r="K24" t="inlineStr">
         <is>
-          <t>I KNOW YOU</t>
+          <t>JIB Official Store</t>
         </is>
       </c>
       <c r="L24" t="n">
@@ -1713,22 +1695,27 @@
           <t>item</t>
         </is>
       </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>5090</t>
+        </is>
+      </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>คอมประกอบพรีเมียม / 4K | Ryzen 9 9950X3D + RTX 5090 32GB | DDR5 32GB / SSD 1TB | พร้อมใช้ ประกันไทย</t>
+          <t>คอมประกอบ GIGABYTE AITOP : Computer Set intel #i375 ULTRA 9 285K RTX5090 32GB GIGABYTE WINDFORCE (OC/D7) - A0172192</t>
         </is>
       </c>
       <c r="E25" t="n">
-        <v>204900</v>
+        <v>301100</v>
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/qhdgLeUAN</t>
+          <t>https://s.shopee.co.th/1gGkfsbJTQ</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>https://down-bs-th.img.susercontent.com/th-11134207-81ztd-mpx5tygok26833.webp</t>
+          <t>https://down-zl-th.img.susercontent.com/th-11134207-81ztn-mq8t04g63tvx56.webp</t>
         </is>
       </c>
       <c r="I25" t="inlineStr">
@@ -1743,7 +1730,7 @@
       </c>
       <c r="K25" t="inlineStr">
         <is>
-          <t>บริษัท มังกี้ อีทีซี. จำกัด</t>
+          <t>Advice Official Shop</t>
         </is>
       </c>
     </row>
@@ -1758,22 +1745,27 @@
           <t>item</t>
         </is>
       </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>5090</t>
+        </is>
+      </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>คอมประกอบพรีเมียม / 4K | Ryzen 7 9800X3D + RTX 5090 32GB | DDR5 32GB / SSD 1TB | พร้อมใช้ ประกันไทย</t>
+          <t>คอมประกอบพรีเมียม / 4K | Ryzen 9 9950X3D + RTX 5090 | DDR5 12GB 6000MHz / SSD 1TB | ชุดน้ำปิด</t>
         </is>
       </c>
       <c r="E26" t="n">
-        <v>193900</v>
+        <v>236900</v>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/LlN5QgOBI</t>
+          <t>https://s.shopee.co.th/1qaAsBag8T</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>https://down-bs-th.img.susercontent.com/th-11134207-81ztd-mpx5tygok26833.webp</t>
+          <t>https://down-zl-th.img.susercontent.com/sg-11134275-821eo-mh0e5nskf7k86e.webp</t>
         </is>
       </c>
       <c r="I26" t="inlineStr">
@@ -1803,22 +1795,27 @@
           <t>item</t>
         </is>
       </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>5090</t>
+        </is>
+      </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>ASUS VGA GEFORCE RTX 5090 ROG ASTRAL O32G GAMING WHITE - 32GB GDDR7 - A0177699</t>
+          <t>GIGABYTE RTX5090 AORUS INFINITY 32GB GDDR7</t>
         </is>
       </c>
       <c r="E27" t="n">
-        <v>205600</v>
+        <v>288900</v>
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/W4nHjfkqL</t>
+          <t>https://s.shopee.co.th/1LduHGca9O</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>https://down-bs-th.img.susercontent.com/sg-11134275-825zz-mkf6jms5jdhgb4.webp</t>
+          <t>https://down-zl-th.img.susercontent.com/th-11134207-81zte-mpeku3c4tngscb.webp</t>
         </is>
       </c>
       <c r="I27" t="inlineStr">
@@ -1833,7 +1830,7 @@
       </c>
       <c r="K27" t="inlineStr">
         <is>
-          <t>Advice Official Shop</t>
+          <t>EXPERT MINES COMPANY LIMITED</t>
         </is>
       </c>
     </row>
@@ -1848,22 +1845,27 @@
           <t>item</t>
         </is>
       </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>5090</t>
+        </is>
+      </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>คอมประกอบพรีเมียม / 4K | Ryzen 7 9800X3D + RTX 5090 | DDR5 12GB / SSD 1TB | ชุดน้ำปิด</t>
+          <t>MSI RTX5090 SUPRIM SOC 32GB GDDR7</t>
         </is>
       </c>
       <c r="E28" t="n">
-        <v>193400</v>
+        <v>195500</v>
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/18WgoherG</t>
+          <t>https://s.shopee.co.th/1VxKTZbwoR</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>https://down-bs-th.img.susercontent.com/th-11134207-81ztc-mpxe9accfaq525.webp</t>
+          <t>https://down-zl-th.img.susercontent.com/th-11134207-7ras8-m8fwept4cfgvaf.webp</t>
         </is>
       </c>
       <c r="I28" t="inlineStr">
@@ -1878,8 +1880,11 @@
       </c>
       <c r="K28" t="inlineStr">
         <is>
-          <t>บริษัท มังกี้ อีทีซี. จำกัด</t>
-        </is>
+          <t>EXPERT MINES COMPANY LIMITED</t>
+        </is>
+      </c>
+      <c r="L28" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="29">
@@ -1893,22 +1898,27 @@
           <t>item</t>
         </is>
       </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>5090</t>
+        </is>
+      </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>MSI RTX5090 GAMING TRIO OC 32GB GDDR7</t>
+          <t>VGA (การ์ดแสดงผล) ASUS ROG ASTRAL GEFORCE RTX 5090 32GB GDDR7 OC EDITION</t>
         </is>
       </c>
       <c r="E29" t="n">
-        <v>189900</v>
+        <v>180700</v>
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/BRwt7h1WJ</t>
+          <t>https://s.shopee.co.th/1113sedqpM</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>https://down-bs-th.img.susercontent.com/th-11134207-81ztg-mipnxvm0gi69ef.webp</t>
+          <t>https://down-zl-th.img.susercontent.com/th-11134207-7ra0u-mb7sojhocgfq48.webp</t>
         </is>
       </c>
       <c r="I29" t="inlineStr">
@@ -1923,7 +1933,7 @@
       </c>
       <c r="K29" t="inlineStr">
         <is>
-          <t>EXPERT MINES COMPANY LIMITED</t>
+          <t>JIB Official Store</t>
         </is>
       </c>
     </row>
@@ -1938,22 +1948,27 @@
           <t>item</t>
         </is>
       </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>5090</t>
+        </is>
+      </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>ASUS ROG ASTRAL RTX5090 GAMING OC WHITE EDITION 32GB GDDR7</t>
+          <t>ASUS ROG ASTRAL GAMING GEFORCE RTX5090 OC EDITION /32GB GDDR7 (90YV0LW0-M0NA00)</t>
         </is>
       </c>
       <c r="E30" t="n">
-        <v>198500</v>
+        <v>180000</v>
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/50XCe0OciG</t>
+          <t>https://s.shopee.co.th/1BKU4xdDUP</t>
         </is>
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>https://down-bs-th.img.susercontent.com/th-11134207-81zto-mibay3dbo0lf65.webp</t>
+          <t>https://down-zl-th.img.susercontent.com/th-11134207-7rasb-m847by4n5tkec6.webp</t>
         </is>
       </c>
       <c r="I30" t="inlineStr">
@@ -1968,8 +1983,11 @@
       </c>
       <c r="K30" t="inlineStr">
         <is>
-          <t>EXPERT MINES COMPANY LIMITED</t>
-        </is>
+          <t>TECHNOCOM.OFFICIAL</t>
+        </is>
+      </c>
+      <c r="L30" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="31">
@@ -1983,22 +2001,27 @@
           <t>item</t>
         </is>
       </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>5090</t>
+        </is>
+      </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>AORUS RTX5090 EXTREME WATERFORCE WB 32GB GDDR7</t>
+          <t>ASUS RTX 5090 ระบบระบายความร้อนด้วยน้ำ Night God Wind Cooling Night God TUF ZTE PowerColor 5090 OC เวอร์ชันต่างประเทศ</t>
         </is>
       </c>
       <c r="E31" t="n">
-        <v>189000</v>
+        <v>337700</v>
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/5AqcqJNzNJ</t>
+          <t>https://s.shopee.co.th/gODU2f7VK</t>
         </is>
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>https://down-bs-th.img.susercontent.com/th-11134207-81ztj-mf53ayfgm3nza4.webp</t>
+          <t>https://down-zl-th.img.susercontent.com/sg-11134201-8260c-mk0ukmy20v7p69.webp</t>
         </is>
       </c>
       <c r="I31" t="inlineStr">
@@ -2013,8 +2036,11 @@
       </c>
       <c r="K31" t="inlineStr">
         <is>
-          <t>EXPERT MINES COMPANY LIMITED</t>
-        </is>
+          <t>I KNOW YOU</t>
+        </is>
+      </c>
+      <c r="L31" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="32">
@@ -2028,22 +2054,27 @@
           <t>item</t>
         </is>
       </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>5090</t>
+        </is>
+      </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>ROG ASTRAL RTX5090 OC 32GB GDDR7</t>
+          <t>คอมประกอบพรีเมียม / 4K | Ryzen 9 9950X3D + RTX 5090 32GB | DDR5 32GB / SSD 1TB | พร้อมใช้ ประกันไทย</t>
         </is>
       </c>
       <c r="E32" t="n">
-        <v>192900</v>
+        <v>204900</v>
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/4fuMFOPtOE</t>
+          <t>https://s.shopee.co.th/qhdgLeUAN</t>
         </is>
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>https://down-bs-th.img.susercontent.com/th-11134207-81ztf-mlolokuve51ra9.webp</t>
+          <t>https://down-bs-th.img.susercontent.com/th-11134207-81ztd-mpx5tygok26833.webp</t>
         </is>
       </c>
       <c r="I32" t="inlineStr">
@@ -2058,7 +2089,7 @@
       </c>
       <c r="K32" t="inlineStr">
         <is>
-          <t>EXPERT MINES COMPANY LIMITED</t>
+          <t>บริษัท มังกี้ อีทีซี. จำกัด</t>
         </is>
       </c>
     </row>
@@ -2073,22 +2104,27 @@
           <t>item</t>
         </is>
       </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>5090</t>
+        </is>
+      </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>GIGABYTE RTX5090 WINDFORCE OC 32GB GDDR7</t>
+          <t>คอมประกอบพรีเมียม / 4K | Ryzen 7 9800X3D + RTX 5090 32GB | DDR5 32GB / SSD 1TB | พร้อมใช้ ประกันไทย</t>
         </is>
       </c>
       <c r="E33" t="n">
-        <v>187900</v>
+        <v>193900</v>
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/4qDmRhPG3H</t>
+          <t>https://s.shopee.co.th/LlN5QgOBI</t>
         </is>
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>https://down-bs-th.img.susercontent.com/th-11134207-7rasf-m8x6avrr1sztc8.webp</t>
+          <t>https://down-bs-th.img.susercontent.com/th-11134207-81ztd-mpx5tygok26833.webp</t>
         </is>
       </c>
       <c r="I33" t="inlineStr">
@@ -2103,7 +2139,7 @@
       </c>
       <c r="K33" t="inlineStr">
         <is>
-          <t>EXPERT MINES COMPANY LIMITED</t>
+          <t>บริษัท มังกี้ อีทีซี. จำกัด</t>
         </is>
       </c>
     </row>
@@ -2118,22 +2154,27 @@
           <t>item</t>
         </is>
       </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>5090</t>
+        </is>
+      </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>ASUS ROG ASTRAL RTX5090 32GB OC GDDR7</t>
+          <t>ASUS VGA GEFORCE RTX 5090 ROG ASTRAL O32G GAMING WHITE - 32GB GDDR7 - A0177699</t>
         </is>
       </c>
       <c r="E34" t="n">
-        <v>198500</v>
+        <v>205600</v>
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/4LHVqmRA4C</t>
+          <t>https://s.shopee.co.th/W4nHjfkqL</t>
         </is>
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>https://down-bs-th.img.susercontent.com/th-11134207-7rase-m76f4vi99o1j85.webp</t>
+          <t>https://down-bs-th.img.susercontent.com/sg-11134275-825zz-mkf6jms5jdhgb4.webp</t>
         </is>
       </c>
       <c r="I34" t="inlineStr">
@@ -2148,11 +2189,8 @@
       </c>
       <c r="K34" t="inlineStr">
         <is>
-          <t>EXPERT MINES COMPANY LIMITED</t>
-        </is>
-      </c>
-      <c r="L34" t="n">
-        <v>3</v>
+          <t>Advice Official Shop</t>
+        </is>
       </c>
     </row>
     <row r="35">
@@ -2166,22 +2204,27 @@
           <t>item</t>
         </is>
       </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>5090</t>
+        </is>
+      </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>GIGABYTE RTX5090 AORUS MASTER 32GB GDDR7</t>
+          <t>คอมประกอบพรีเมียม / 4K | Ryzen 7 9800X3D + RTX 5090 | DDR5 12GB / SSD 1TB | ชุดน้ำปิด</t>
         </is>
       </c>
       <c r="E35" t="n">
-        <v>195500</v>
+        <v>193400</v>
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/4Vaw35QWjF</t>
+          <t>https://s.shopee.co.th/18WgoherG</t>
         </is>
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>https://down-bs-th.img.susercontent.com/th-11134207-7rash-m8x6kptwxcgf32.webp</t>
+          <t>https://down-bs-th.img.susercontent.com/th-11134207-81ztc-mpxe9accfaq525.webp</t>
         </is>
       </c>
       <c r="I35" t="inlineStr">
@@ -2196,7 +2239,7 @@
       </c>
       <c r="K35" t="inlineStr">
         <is>
-          <t>EXPERT MINES COMPANY LIMITED</t>
+          <t>บริษัท มังกี้ อีทีซี. จำกัด</t>
         </is>
       </c>
     </row>
@@ -2211,22 +2254,27 @@
           <t>item</t>
         </is>
       </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>5090</t>
+        </is>
+      </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>คอมพิวเตอร์ประกอบ THERMALTAKE TOWER 600 RTX5090 ASTRAL LC ULTRA 9 285K BLACK</t>
+          <t>MSI RTX5090 GAMING TRIO OC 32GB GDDR7</t>
         </is>
       </c>
       <c r="E36" t="n">
-        <v>459500</v>
+        <v>189900</v>
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/40efSASQkA</t>
+          <t>https://s.shopee.co.th/BRwt7h1WJ</t>
         </is>
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>https://down-bs-th.img.susercontent.com/th-11134207-7rasg-m8vrk1wnfevde1.webp</t>
+          <t>https://down-bs-th.img.susercontent.com/th-11134207-81ztg-mipnxvm0gi69ef.webp</t>
         </is>
       </c>
       <c r="I36" t="inlineStr">
@@ -2256,22 +2304,27 @@
           <t>item</t>
         </is>
       </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>5090</t>
+        </is>
+      </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>ZOTAC RTX5090 SOLID GAMING OC WHITE 32GB GDDR7</t>
+          <t>ASUS ROG ASTRAL RTX5090 GAMING OC WHITE EDITION 32GB GDDR7</t>
         </is>
       </c>
       <c r="E37" t="n">
-        <v>186900</v>
+        <v>198500</v>
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/4Ay5eTRnPD</t>
+          <t>https://s.shopee.co.th/50XCe0OciG</t>
         </is>
       </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t>https://down-bs-th.img.susercontent.com/th-11134207-7ras8-m8eac2h34cnd54.webp</t>
+          <t>https://down-bs-th.img.susercontent.com/th-11134207-81zto-mibay3dbo0lf65.webp</t>
         </is>
       </c>
       <c r="I37" t="inlineStr">
@@ -2301,22 +2354,27 @@
           <t>item</t>
         </is>
       </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>5090</t>
+        </is>
+      </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>ZOTAC GAMING RTX5090 SOLID OC 32GB GDDR7</t>
+          <t>AORUS RTX5090 EXTREME WATERFORCE WB 32GB GDDR7</t>
         </is>
       </c>
       <c r="E38" t="n">
-        <v>186900</v>
+        <v>189000</v>
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/3g1p3YThQ8</t>
+          <t>https://s.shopee.co.th/5AqcqJNzNJ</t>
         </is>
       </c>
       <c r="H38" t="inlineStr">
         <is>
-          <t>https://down-bs-th.img.susercontent.com/th-11134207-81zth-mlogm2dcg5j558.webp</t>
+          <t>https://down-bs-th.img.susercontent.com/th-11134207-81ztj-mf53ayfgm3nza4.webp</t>
         </is>
       </c>
       <c r="I38" t="inlineStr">
@@ -2346,22 +2404,27 @@
           <t>item</t>
         </is>
       </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>5090</t>
+        </is>
+      </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>[สินค้าพร้อมจัดส่งในไทย] GIGABYTE GAMING RTX5090 32GB GDDR7 OC EDITION</t>
+          <t>ROG ASTRAL RTX5090 OC 32GB GDDR7</t>
         </is>
       </c>
       <c r="E39" t="n">
-        <v>185500</v>
+        <v>192900</v>
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/3qLFFrT45B</t>
+          <t>https://s.shopee.co.th/4fuMFOPtOE</t>
         </is>
       </c>
       <c r="H39" t="inlineStr">
         <is>
-          <t>https://down-bs-th.img.susercontent.com/th-11134207-7rase-m6r6xy11sncf25.webp</t>
+          <t>https://down-bs-th.img.susercontent.com/th-11134207-81ztf-mlolokuve51ra9.webp</t>
         </is>
       </c>
       <c r="I39" t="inlineStr">
@@ -2391,22 +2454,27 @@
           <t>item</t>
         </is>
       </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>5090</t>
+        </is>
+      </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>MSI RTX5090 32G LIGHTNING Z GDDR7</t>
+          <t>GIGABYTE RTX5090 WINDFORCE OC 32GB GDDR7</t>
         </is>
       </c>
       <c r="E40" t="n">
-        <v>269500</v>
+        <v>187900</v>
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/3LOyewUy66</t>
+          <t>https://s.shopee.co.th/4qDmRhPG3H</t>
         </is>
       </c>
       <c r="H40" t="inlineStr">
         <is>
-          <t>https://down-bs-th.img.susercontent.com/th-11134207-81ztp-mlisa7sidtdw15.webp</t>
+          <t>https://down-bs-th.img.susercontent.com/th-11134207-7rasf-m8x6avrr1sztc8.webp</t>
         </is>
       </c>
       <c r="I40" t="inlineStr">
@@ -2436,22 +2504,27 @@
           <t>item</t>
         </is>
       </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>5090</t>
+        </is>
+      </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>GIGABYTE AORUS RTX5090 STEALTH ICE 32GB GDDR7</t>
+          <t>ASUS ROG ASTRAL RTX5090 32GB OC GDDR7</t>
         </is>
       </c>
       <c r="E41" t="n">
-        <v>195000</v>
+        <v>198500</v>
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/3ViOrFUKl9</t>
+          <t>https://s.shopee.co.th/4LHVqmRA4C</t>
         </is>
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t>https://down-bs-th.img.susercontent.com/th-11134207-7ra0g-mczwcxljswclad.webp</t>
+          <t>https://down-bs-th.img.susercontent.com/th-11134207-7rase-m76f4vi99o1j85.webp</t>
         </is>
       </c>
       <c r="I41" t="inlineStr">
@@ -2468,6 +2541,9 @@
         <is>
           <t>EXPERT MINES COMPANY LIMITED</t>
         </is>
+      </c>
+      <c r="L41" t="n">
+        <v>3</v>
       </c>
     </row>
     <row r="42">
@@ -2481,9 +2557,14 @@
           <t>item</t>
         </is>
       </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>5090</t>
+        </is>
+      </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>GIGABYTE RTX5090 AORUS MASTER ICE GDDR7</t>
+          <t>GIGABYTE RTX5090 AORUS MASTER 32GB GDDR7</t>
         </is>
       </c>
       <c r="E42" t="n">
@@ -2491,12 +2572,12 @@
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/30m8GKWEm4</t>
+          <t>https://s.shopee.co.th/4Vaw35QWjF</t>
         </is>
       </c>
       <c r="H42" t="inlineStr">
         <is>
-          <t>https://down-bs-th.img.susercontent.com/th-11134207-81ztq-mdzlhtv1g2yo1b.webp</t>
+          <t>https://down-bs-th.img.susercontent.com/th-11134207-7rash-m8x6kptwxcgf32.webp</t>
         </is>
       </c>
       <c r="I42" t="inlineStr">
@@ -2526,22 +2607,27 @@
           <t>item</t>
         </is>
       </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>5090</t>
+        </is>
+      </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>INNO3D RTX5090 ICHILL X3 32GB OC GDDR7</t>
+          <t>คอมพิวเตอร์ประกอบ THERMALTAKE TOWER 600 RTX5090 ASTRAL LC ULTRA 9 285K BLACK</t>
         </is>
       </c>
       <c r="E43" t="n">
-        <v>179900</v>
+        <v>459500</v>
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/3B5YSdVbR7</t>
+          <t>https://s.shopee.co.th/40efSASQkA</t>
         </is>
       </c>
       <c r="H43" t="inlineStr">
         <is>
-          <t>https://down-bs-th.img.susercontent.com/th-11134207-7rasd-m8eajig8ywaxe9.webp</t>
+          <t>https://down-bs-th.img.susercontent.com/th-11134207-7rasg-m8vrk1wnfevde1.webp</t>
         </is>
       </c>
       <c r="I43" t="inlineStr">
@@ -2571,22 +2657,27 @@
           <t>item</t>
         </is>
       </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>5090</t>
+        </is>
+      </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>[สินค้าพร้อมจัดส่งในไทย] ASUS TUF GAMING RTX5090 32GB GDDR7</t>
+          <t>ZOTAC RTX5090 SOLID GAMING OC WHITE 32GB GDDR7</t>
         </is>
       </c>
       <c r="E44" t="n">
-        <v>185500</v>
+        <v>186900</v>
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/2g9HriXVS2</t>
+          <t>https://s.shopee.co.th/4Ay5eTRnPD</t>
         </is>
       </c>
       <c r="H44" t="inlineStr">
         <is>
-          <t>https://down-bs-th.img.susercontent.com/th-11134207-7rasd-m8x5qjjikva8b0.webp</t>
+          <t>https://down-bs-th.img.susercontent.com/th-11134207-7ras8-m8eac2h34cnd54.webp</t>
         </is>
       </c>
       <c r="I44" t="inlineStr">
@@ -2616,22 +2707,27 @@
           <t>item</t>
         </is>
       </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>5090</t>
+        </is>
+      </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>ASUS ROG ASTRAL RTX5090 GAMING OC BTF 32GB GDDR7</t>
+          <t>ZOTAC GAMING RTX5090 SOLID OC 32GB GDDR7</t>
         </is>
       </c>
       <c r="E45" t="n">
-        <v>198500</v>
+        <v>186900</v>
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/2qSi41Ws75</t>
+          <t>https://s.shopee.co.th/3g1p3YThQ8</t>
         </is>
       </c>
       <c r="H45" t="inlineStr">
         <is>
-          <t>https://down-bs-th.img.susercontent.com/th-11134207-81ztd-mnjoolkkmxoldd.webp</t>
+          <t>https://down-bs-th.img.susercontent.com/th-11134207-81zth-mlogm2dcg5j558.webp</t>
         </is>
       </c>
       <c r="I45" t="inlineStr">
@@ -2661,22 +2757,27 @@
           <t>item</t>
         </is>
       </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>5090</t>
+        </is>
+      </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>MSI RTX5090 32GB VENTUS 3X OC GDDR7</t>
+          <t>[สินค้าพร้อมจัดส่งในไทย] GIGABYTE GAMING RTX5090 32GB GDDR7 OC EDITION</t>
         </is>
       </c>
       <c r="E46" t="n">
-        <v>192900</v>
+        <v>185500</v>
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/7fXxouETJ2</t>
+          <t>https://s.shopee.co.th/3qLFFrT45B</t>
         </is>
       </c>
       <c r="H46" t="inlineStr">
         <is>
-          <t>https://down-bs-th.img.susercontent.com/th-11134207-7rasl-m8d2dtf6q4mm9d.webp</t>
+          <t>https://down-bs-th.img.susercontent.com/th-11134207-7rase-m6r6xy11sncf25.webp</t>
         </is>
       </c>
       <c r="I46" t="inlineStr">
@@ -2706,22 +2807,27 @@
           <t>item</t>
         </is>
       </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>5090</t>
+        </is>
+      </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>ZOTAC RTX5090 AMP EXTREME INFINITY 32GB GDDR7</t>
+          <t>MSI RTX5090 32G LIGHTNING Z GDDR7</t>
         </is>
       </c>
       <c r="E47" t="n">
-        <v>188500</v>
+        <v>269500</v>
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/7prO1DDpy5</t>
+          <t>https://s.shopee.co.th/3LOyewUy66</t>
         </is>
       </c>
       <c r="H47" t="inlineStr">
         <is>
-          <t>https://down-bs-th.img.susercontent.com/th-11134207-7rasa-m5js2fig00fea0.webp</t>
+          <t>https://down-bs-th.img.susercontent.com/th-11134207-81ztp-mlisa7sidtdw15.webp</t>
         </is>
       </c>
       <c r="I47" t="inlineStr">
@@ -2751,22 +2857,27 @@
           <t>item</t>
         </is>
       </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>5090</t>
+        </is>
+      </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>ASUS ROG ASTRAL LC RTX5090 32GB OC GDDR7</t>
+          <t>GIGABYTE AORUS RTX5090 STEALTH ICE 32GB GDDR7</t>
         </is>
       </c>
       <c r="E48" t="n">
-        <v>215000</v>
+        <v>195000</v>
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/7Kv7QIFjz0</t>
+          <t>https://s.shopee.co.th/3ViOrFUKl9</t>
         </is>
       </c>
       <c r="H48" t="inlineStr">
         <is>
-          <t>https://down-bs-th.img.susercontent.com/th-11134207-7rasa-m5js2fig00fea0.webp</t>
+          <t>https://down-bs-th.img.susercontent.com/th-11134207-7ra0g-mczwcxljswclad.webp</t>
         </is>
       </c>
       <c r="I48" t="inlineStr">
@@ -2796,22 +2907,27 @@
           <t>item</t>
         </is>
       </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>5090</t>
+        </is>
+      </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>VGA (การ์ดแสดงผล) MSI GEFORCE RTX 5090 32G LIGHTNING Z - 32GB GDDR7</t>
+          <t>GIGABYTE RTX5090 AORUS MASTER ICE GDDR7</t>
         </is>
       </c>
       <c r="E49" t="n">
-        <v>228800</v>
+        <v>195500</v>
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/7VEXcbF6e3</t>
+          <t>https://s.shopee.co.th/30m8GKWEm4</t>
         </is>
       </c>
       <c r="H49" t="inlineStr">
         <is>
-          <t>https://down-bs-th.img.susercontent.com/th-11134207-7rasd-m7j5dkasn5qyce.webp</t>
+          <t>https://down-bs-th.img.susercontent.com/th-11134207-81ztq-mdzlhtv1g2yo1b.webp</t>
         </is>
       </c>
       <c r="I49" t="inlineStr">
@@ -2826,7 +2942,7 @@
       </c>
       <c r="K49" t="inlineStr">
         <is>
-          <t>JIB Official Store</t>
+          <t>EXPERT MINES COMPANY LIMITED</t>
         </is>
       </c>
     </row>
@@ -2841,22 +2957,27 @@
           <t>item</t>
         </is>
       </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>5090</t>
+        </is>
+      </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>GIGABYTE GEFORCE RTX 5090 GAMING OC 32G – 32GB GDDR7 (GV-N5090GAMING OC-32GD) (ALI) (TBO-15 Days)</t>
+          <t>INNO3D RTX5090 ICHILL X3 32GB OC GDDR7</t>
         </is>
       </c>
       <c r="E50" t="n">
-        <v>209000</v>
+        <v>179900</v>
       </c>
       <c r="G50" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/70IH1gH0ey</t>
+          <t>https://s.shopee.co.th/3B5YSdVbR7</t>
         </is>
       </c>
       <c r="H50" t="inlineStr">
         <is>
-          <t>https://down-bs-th.img.susercontent.com/th-11134207-81zti-mllhvztzby0w0e.webp</t>
+          <t>https://down-bs-th.img.susercontent.com/th-11134207-7rasd-m8eajig8ywaxe9.webp</t>
         </is>
       </c>
       <c r="I50" t="inlineStr">
@@ -2871,7 +2992,7 @@
       </c>
       <c r="K50" t="inlineStr">
         <is>
-          <t>shoppingpc dotnet</t>
+          <t>EXPERT MINES COMPANY LIMITED</t>
         </is>
       </c>
     </row>
@@ -2886,17 +3007,27 @@
           <t>item</t>
         </is>
       </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>5090</t>
+        </is>
+      </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>การ์ดจอ RTX 3060Ti 3060Ti 4060 4070 4080 5070 5080 5090</t>
+          <t>[สินค้าพร้อมจัดส่งในไทย] ASUS TUF GAMING RTX5090 32GB GDDR7</t>
         </is>
       </c>
       <c r="E51" t="n">
-        <v>9000</v>
+        <v>185500</v>
       </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/7AbhDzGNK1</t>
+          <t>https://s.shopee.co.th/2g9HriXVS2</t>
+        </is>
+      </c>
+      <c r="H51" t="inlineStr">
+        <is>
+          <t>https://down-bs-th.img.susercontent.com/th-11134207-7rasd-m8x5qjjikva8b0.webp</t>
         </is>
       </c>
       <c r="I51" t="inlineStr">
@@ -2911,17 +3042,14 @@
       </c>
       <c r="K51" t="inlineStr">
         <is>
-          <t>EZGGTECH</t>
-        </is>
-      </c>
-      <c r="L51" t="n">
-        <v>1</v>
+          <t>EXPERT MINES COMPANY LIMITED</t>
+        </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>ai_calculator_cpu</t>
+          <t>ai_calculator</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
@@ -2929,23 +3057,27 @@
           <t>item</t>
         </is>
       </c>
-      <c r="C52" t="inlineStr"/>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>5090</t>
+        </is>
+      </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>CPU (ซีพียู) AMD RYZEN 9 7950X 4.5 GHz (SOCKET AM5) (ระบบระบายความร้อนไม่รวมอยู่ในสินค้า) -3 YEARS</t>
+          <t>ASUS ROG ASTRAL RTX5090 GAMING OC BTF 32GB GDDR7</t>
         </is>
       </c>
       <c r="E52" t="n">
-        <v>22700</v>
+        <v>198500</v>
       </c>
       <c r="G52" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/2qSiUqO1NA</t>
+          <t>https://s.shopee.co.th/2qSi41Ws75</t>
         </is>
       </c>
       <c r="H52" t="inlineStr">
         <is>
-          <t>https://down-ws-th.img.susercontent.com/th-11134207-7rasd-m8x801x6gycuda.webp</t>
+          <t>https://down-bs-th.img.susercontent.com/th-11134207-81ztd-mnjoolkkmxoldd.webp</t>
         </is>
       </c>
       <c r="I52" t="inlineStr">
@@ -2953,19 +3085,21 @@
           <t>Shopee</t>
         </is>
       </c>
+      <c r="J52" t="inlineStr">
+        <is>
+          <t>ขายดี</t>
+        </is>
+      </c>
       <c r="K52" t="inlineStr">
         <is>
-          <t>mcwinner</t>
-        </is>
-      </c>
-      <c r="L52" t="n">
-        <v>19</v>
+          <t>EXPERT MINES COMPANY LIMITED</t>
+        </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>ai_calculator_cpu</t>
+          <t>ai_calculator</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
@@ -2973,23 +3107,27 @@
           <t>item</t>
         </is>
       </c>
-      <c r="C53" t="inlineStr"/>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>5090</t>
+        </is>
+      </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>CPU (ซีพียู) AMD RYZEN 9 9950X - 16C 32T 4.3-5.7GHz (AMD SOCKET AM5) (ระบบระบายความร้อนไม่รวมอยู่ในสินค้า)</t>
+          <t>MSI RTX5090 32GB VENTUS 3X OC GDDR7</t>
         </is>
       </c>
       <c r="E53" t="n">
-        <v>26500</v>
+        <v>192900</v>
       </c>
       <c r="G53" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/2g9IIXOei9</t>
+          <t>https://s.shopee.co.th/7fXxouETJ2</t>
         </is>
       </c>
       <c r="H53" t="inlineStr">
         <is>
-          <t>https://down-ws-th.img.susercontent.com/th-11134207-7r991-m08fblrkcqfsb1.webp</t>
+          <t>https://down-bs-th.img.susercontent.com/th-11134207-7rasl-m8d2dtf6q4mm9d.webp</t>
         </is>
       </c>
       <c r="I53" t="inlineStr">
@@ -2997,19 +3135,21 @@
           <t>Shopee</t>
         </is>
       </c>
+      <c r="J53" t="inlineStr">
+        <is>
+          <t>ขายดี</t>
+        </is>
+      </c>
       <c r="K53" t="inlineStr">
         <is>
-          <t>JIB Official Store</t>
-        </is>
-      </c>
-      <c r="L53" t="n">
-        <v>6</v>
+          <t>EXPERT MINES COMPANY LIMITED</t>
+        </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>ai_calculator_cpu</t>
+          <t>ai_calculator</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
@@ -3017,23 +3157,27 @@
           <t>item</t>
         </is>
       </c>
-      <c r="C54" t="inlineStr"/>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>5090</t>
+        </is>
+      </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>CPU (ซีพียู) AMD RYZEN 5 9600X - 6C 12T 3.9-5.4GHz (AMD SOCKET AM5) (ระบบระบายความร้อนไม่รวมอยู่ในสินค้า)</t>
+          <t>ZOTAC RTX5090 AMP EXTREME INFINITY 32GB GDDR7</t>
         </is>
       </c>
       <c r="E54" t="n">
-        <v>10500</v>
+        <v>188500</v>
       </c>
       <c r="G54" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/3B5YtSMkhG</t>
+          <t>https://s.shopee.co.th/7prO1DDpy5</t>
         </is>
       </c>
       <c r="H54" t="inlineStr">
         <is>
-          <t>https://down-ws-th.img.susercontent.com/th-11134207-7ras8-m7agd6ph9f744c.webp</t>
+          <t>https://down-bs-th.img.susercontent.com/th-11134207-7rasa-m5js2fig00fea0.webp</t>
         </is>
       </c>
       <c r="I54" t="inlineStr">
@@ -3041,19 +3185,21 @@
           <t>Shopee</t>
         </is>
       </c>
+      <c r="J54" t="inlineStr">
+        <is>
+          <t>ขายดี</t>
+        </is>
+      </c>
       <c r="K54" t="inlineStr">
         <is>
-          <t>JIB Official Store</t>
-        </is>
-      </c>
-      <c r="L54" t="n">
-        <v>382</v>
+          <t>EXPERT MINES COMPANY LIMITED</t>
+        </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>ai_calculator_cpu</t>
+          <t>ai_calculator</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
@@ -3061,23 +3207,27 @@
           <t>item</t>
         </is>
       </c>
-      <c r="C55" t="inlineStr"/>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>5090</t>
+        </is>
+      </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>CPU (ซีพียู) AMD RYZEN 9 9950X3D - 16C 32T 4.3-5.7GHz AMD SOCKET AM5 (ระบบระบายความร้อนไม่รวมอยู่ในสินค้า)</t>
+          <t>ASUS ROG ASTRAL LC RTX5090 32GB OC GDDR7</t>
         </is>
       </c>
       <c r="E55" t="n">
-        <v>33000</v>
+        <v>215000</v>
       </c>
       <c r="G55" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/30m8h9NO2F</t>
+          <t>https://s.shopee.co.th/7Kv7QIFjz0</t>
         </is>
       </c>
       <c r="H55" t="inlineStr">
         <is>
-          <t>https://down-ws-th.img.susercontent.com/th-11134207-7rasd-m8ylj449xemnd8.webp</t>
+          <t>https://down-bs-th.img.susercontent.com/th-11134207-7rasa-m5js2fig00fea0.webp</t>
         </is>
       </c>
       <c r="I55" t="inlineStr">
@@ -3085,19 +3235,21 @@
           <t>Shopee</t>
         </is>
       </c>
+      <c r="J55" t="inlineStr">
+        <is>
+          <t>ขายดี</t>
+        </is>
+      </c>
       <c r="K55" t="inlineStr">
         <is>
-          <t>JIB Official Store</t>
-        </is>
-      </c>
-      <c r="L55" t="n">
-        <v>6</v>
+          <t>EXPERT MINES COMPANY LIMITED</t>
+        </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>ai_calculator_cpu</t>
+          <t>ai_calculator</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
@@ -3105,23 +3257,27 @@
           <t>item</t>
         </is>
       </c>
-      <c r="C56" t="inlineStr"/>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>5090</t>
+        </is>
+      </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>ซีพียู CPU: AMD - RYZEN 9 (9950X AM5)</t>
+          <t>VGA (การ์ดแสดงผล) MSI GEFORCE RTX 5090 32G LIGHTNING Z - 32GB GDDR7</t>
         </is>
       </c>
       <c r="E56" t="n">
-        <v>29900</v>
+        <v>228800</v>
       </c>
       <c r="G56" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/3ViPI4LU1M</t>
+          <t>https://s.shopee.co.th/7VEXcbF6e3</t>
         </is>
       </c>
       <c r="H56" t="inlineStr">
         <is>
-          <t>https://down-ws-th.img.susercontent.com/th-11134275-7rasm-maw7h34vstcg33.webp</t>
+          <t>https://down-bs-th.img.susercontent.com/th-11134207-7rasd-m7j5dkasn5qyce.webp</t>
         </is>
       </c>
       <c r="I56" t="inlineStr">
@@ -3129,19 +3285,21 @@
           <t>Shopee</t>
         </is>
       </c>
+      <c r="J56" t="inlineStr">
+        <is>
+          <t>ขายดี</t>
+        </is>
+      </c>
       <c r="K56" t="inlineStr">
         <is>
-          <t>atSine Tech</t>
-        </is>
-      </c>
-      <c r="L56" t="n">
-        <v>2</v>
+          <t>JIB Official Store</t>
+        </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>ai_calculator_cpu</t>
+          <t>ai_calculator</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
@@ -3149,23 +3307,27 @@
           <t>item</t>
         </is>
       </c>
-      <c r="C57" t="inlineStr"/>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>5090</t>
+        </is>
+      </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>CPU AMD AM5 RYZEN 9 9900X3D (NEXT) - A0169017</t>
+          <t>GIGABYTE GEFORCE RTX 5090 GAMING OC 32G – 32GB GDDR7 (GV-N5090GAMING OC-32GD) (ALI) (TBO-15 Days)</t>
         </is>
       </c>
       <c r="E57" t="n">
-        <v>24200</v>
+        <v>209000</v>
       </c>
       <c r="G57" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/3LOz5lM7ML</t>
+          <t>https://s.shopee.co.th/70IH1gH0ey</t>
         </is>
       </c>
       <c r="H57" t="inlineStr">
         <is>
-          <t>https://down-ws-th.img.susercontent.com/th-11134275-7rasf-maw7gzrwpuo1b1.webp</t>
+          <t>https://down-bs-th.img.susercontent.com/th-11134207-81zti-mllhvztzby0w0e.webp</t>
         </is>
       </c>
       <c r="I57" t="inlineStr">
@@ -3173,19 +3335,21 @@
           <t>Shopee</t>
         </is>
       </c>
+      <c r="J57" t="inlineStr">
+        <is>
+          <t>ขายดี</t>
+        </is>
+      </c>
       <c r="K57" t="inlineStr">
         <is>
-          <t>Advice Official Shop</t>
-        </is>
-      </c>
-      <c r="L57" t="n">
-        <v>4</v>
+          <t>shoppingpc dotnet</t>
+        </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>ai_calculator_cpu</t>
+          <t>ai_calculator</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
@@ -3193,23 +3357,22 @@
           <t>item</t>
         </is>
       </c>
-      <c r="C58" t="inlineStr"/>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>5090</t>
+        </is>
+      </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>CPU AMD AM5 RYZEN 9 9950X3D (NEXT) - A0168684</t>
+          <t>การ์ดจอ RTX 3060Ti 3060Ti 4060 4070 4080 5070 5080 5090</t>
         </is>
       </c>
       <c r="E58" t="n">
-        <v>32200</v>
+        <v>9000</v>
       </c>
       <c r="G58" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/3qLFggKDLS</t>
-        </is>
-      </c>
-      <c r="H58" t="inlineStr">
-        <is>
-          <t>https://down-ws-th.img.susercontent.com/th-11134275-7rasf-maw7gzrwpuo1b1.webp</t>
+          <t>https://s.shopee.co.th/7AbhDzGNK1</t>
         </is>
       </c>
       <c r="I58" t="inlineStr">
@@ -3217,13 +3380,18 @@
           <t>Shopee</t>
         </is>
       </c>
+      <c r="J58" t="inlineStr">
+        <is>
+          <t>ขายดี</t>
+        </is>
+      </c>
       <c r="K58" t="inlineStr">
         <is>
-          <t>Advice Official Shop</t>
+          <t>EZGGTECH</t>
         </is>
       </c>
       <c r="L58" t="n">
-        <v>11</v>
+        <v>1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>